<commit_message>
add new drawing and measurement
</commit_message>
<xml_diff>
--- a/catalog/adaptor/resource_updated.xlsx
+++ b/catalog/adaptor/resource_updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\ManoEng\catalog\adaptor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69994DFF-ADF1-4738-9923-68152F61D44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13628F78-07FF-4D9E-889D-64D5713259D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{039EFAA4-C4D2-4F31-ABF8-5ECCF156DD30}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{039EFAA4-C4D2-4F31-ABF8-5ECCF156DD30}"/>
   </bookViews>
   <sheets>
     <sheet name="2102856" sheetId="2" r:id="rId1"/>
@@ -282,7 +282,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="115">
   <si>
     <t xml:space="preserve">Picture </t>
   </si>
@@ -669,6 +669,13 @@
   </si>
   <si>
     <t>ZF Electronics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+chenjinbing888@hotmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -3201,8 +3208,8 @@
       <c r="C2" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="18">
-        <v>2.81</v>
+      <c r="D2" s="18" t="s">
+        <v>114</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>102</v>
@@ -3280,7 +3287,9 @@
       <c r="D5" s="6">
         <v>0.5</v>
       </c>
-      <c r="E5" s="6"/>
+      <c r="E5" s="18" t="s">
+        <v>113</v>
+      </c>
       <c r="F5" s="19"/>
       <c r="G5" s="13" t="s">
         <v>63</v>

</xml_diff>